<commit_message>
Add university classification feature to ProgramCard and ProgramSection components
</commit_message>
<xml_diff>
--- a/MBA Options_25.09.2025.xlsx
+++ b/MBA Options_25.09.2025.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aksha\Desktop\Kareer Studio\Integrated\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aksha\Desktop\Kareer Studio\CORE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E62B2ABF-59B2-441B-BF1F-32E5A85BBFFF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4F5166-FA26-451C-8B22-BEF09D552A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="43" uniqueCount="34">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="36">
   <si>
     <t>Serial No.</t>
   </si>
@@ -64,9 +64,6 @@
     <t>24 Months</t>
   </si>
   <si>
-    <t>University of East London</t>
-  </si>
-  <si>
     <t>MBA Master of Business Administration (Business Analytics) with Placement Year</t>
   </si>
   <si>
@@ -124,14 +121,23 @@
     <t>USA</t>
   </si>
   <si>
-    <t>University of New York</t>
+    <t>Yale University</t>
+  </si>
+  <si>
+    <t>King's College London</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dartmouth College </t>
+  </si>
+  <si>
+    <t>East London</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4">
+  <fonts count="5">
     <font>
       <sz val="11"/>
       <name val="Calibri"/>
@@ -150,6 +156,11 @@
     <font>
       <sz val="8"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Calibri"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -203,7 +214,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="7">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
@@ -219,6 +230,9 @@
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -529,7 +543,7 @@
         <v>2</v>
       </c>
       <c r="D1" s="5" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E1" s="5" t="s">
         <v>3</v>
@@ -553,16 +567,16 @@
         <v>9</v>
       </c>
       <c r="L1" s="5" t="s">
+        <v>20</v>
+      </c>
+      <c r="M1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="M1" s="5" t="s">
+      <c r="N1" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="N1" s="5" t="s">
+      <c r="O1" s="5" t="s">
         <v>23</v>
-      </c>
-      <c r="O1" s="5" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="2" spans="1:15" s="2" customFormat="1" ht="28.8">
@@ -570,16 +584,16 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="C2" s="6" t="s">
         <v>13</v>
       </c>
-      <c r="C2" s="6" t="s">
+      <c r="D2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="E2" s="4" t="s">
         <v>15</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>16</v>
       </c>
       <c r="F2" s="4" t="s">
         <v>10</v>
@@ -594,10 +608,10 @@
         <v>6</v>
       </c>
       <c r="J2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K2" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="K2" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="L2" s="4">
         <v>23</v>
@@ -606,7 +620,7 @@
         <v>5</v>
       </c>
       <c r="N2" s="4" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="O2" s="4">
         <v>78</v>
@@ -617,16 +631,16 @@
         <v>2</v>
       </c>
       <c r="B3" s="4" t="s">
-        <v>13</v>
+        <v>33</v>
       </c>
       <c r="C3" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="4" t="s">
-        <v>18</v>
-      </c>
       <c r="E3" s="4" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="F3" s="4" t="s">
         <v>10</v>
@@ -641,10 +655,10 @@
         <v>6</v>
       </c>
       <c r="J3" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="4" t="s">
         <v>27</v>
-      </c>
-      <c r="K3" s="4" t="s">
-        <v>28</v>
       </c>
       <c r="L3" s="4">
         <v>45</v>
@@ -663,20 +677,20 @@
       <c r="A4" s="4">
         <v>3</v>
       </c>
-      <c r="B4" s="4" t="s">
-        <v>33</v>
+      <c r="B4" s="7" t="s">
+        <v>34</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D4" s="4" t="s">
-        <v>20</v>
-      </c>
       <c r="E4" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F4" s="4" t="s">
         <v>31</v>
-      </c>
-      <c r="F4" s="4" t="s">
-        <v>32</v>
       </c>
       <c r="G4" s="4" t="s">
         <v>11</v>
@@ -688,10 +702,10 @@
         <v>6</v>
       </c>
       <c r="J4" s="4" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="L4" s="4">
         <v>43</v>
@@ -706,22 +720,52 @@
         <v>45</v>
       </c>
     </row>
-    <row r="5" spans="1:15" s="2" customFormat="1">
-      <c r="A5" s="4"/>
-      <c r="B5" s="4"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="4"/>
-      <c r="E5" s="4"/>
-      <c r="F5" s="4"/>
-      <c r="G5" s="4"/>
-      <c r="H5" s="4"/>
-      <c r="I5" s="4"/>
-      <c r="J5" s="4"/>
-      <c r="K5" s="4"/>
-      <c r="L5" s="4"/>
-      <c r="M5" s="4"/>
-      <c r="N5" s="4"/>
-      <c r="O5" s="4"/>
+    <row r="5" spans="1:15" s="2" customFormat="1" ht="28.8">
+      <c r="A5" s="4">
+        <v>4</v>
+      </c>
+      <c r="B5" s="7" t="s">
+        <v>35</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="F5" s="4" t="s">
+        <v>31</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="I5" s="4">
+        <v>6</v>
+      </c>
+      <c r="J5" s="4" t="s">
+        <v>29</v>
+      </c>
+      <c r="K5" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="L5" s="4">
+        <v>43</v>
+      </c>
+      <c r="M5" s="4">
+        <v>34</v>
+      </c>
+      <c r="N5" s="4">
+        <v>34</v>
+      </c>
+      <c r="O5" s="4">
+        <v>45</v>
+      </c>
     </row>
     <row r="6" spans="1:15" s="2" customFormat="1">
       <c r="A6" s="4"/>

</xml_diff>

<commit_message>
Add QS ranking lookup utility
- Implemented a new utility for loading and querying QS university rankings from an Excel file.
- Introduced functions to normalize university names, parse rank values, and cache rankings for efficient lookups.
- Added methods to retrieve QS data and rankings based on university names, supporting both exact and substring matches.
- Included error handling for missing files and unparseable rank values.
</commit_message>
<xml_diff>
--- a/MBA Options_25.09.2025.xlsx
+++ b/MBA Options_25.09.2025.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aksha\Desktop\Kareer Studio\CORE\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8A4F5166-FA26-451C-8B22-BEF09D552A31}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E1E96093-9328-4BD9-A4DD-9987C29061F8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -622,9 +622,7 @@
       <c r="N2" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="O2" s="4">
-        <v>78</v>
-      </c>
+      <c r="O2" s="4"/>
     </row>
     <row r="3" spans="1:15" s="2" customFormat="1" ht="28.8">
       <c r="A3" s="4">
@@ -669,9 +667,7 @@
       <c r="N3" s="4">
         <v>77</v>
       </c>
-      <c r="O3" s="4">
-        <v>435</v>
-      </c>
+      <c r="O3" s="4"/>
     </row>
     <row r="4" spans="1:15" s="2" customFormat="1" ht="28.8">
       <c r="A4" s="4">
@@ -716,9 +712,7 @@
       <c r="N4" s="4">
         <v>34</v>
       </c>
-      <c r="O4" s="4">
-        <v>45</v>
-      </c>
+      <c r="O4" s="4"/>
     </row>
     <row r="5" spans="1:15" s="2" customFormat="1" ht="28.8">
       <c r="A5" s="4">
@@ -763,9 +757,7 @@
       <c r="N5" s="4">
         <v>34</v>
       </c>
-      <c r="O5" s="4">
-        <v>45</v>
-      </c>
+      <c r="O5" s="4"/>
     </row>
     <row r="6" spans="1:15" s="2" customFormat="1">
       <c r="A6" s="4"/>

</xml_diff>